<commit_message>
NRCS rule & data changes
</commit_message>
<xml_diff>
--- a/NRCS/Requirements/NRCS_information_New.xlsx
+++ b/NRCS/Requirements/NRCS_information_New.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tanwin/Documents/GitHub/School_TimeTable/NRCS/Requirements/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A2887E1-D297-C940-9EFF-5D7292F56C2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6ED00339-AEA6-2D40-8D86-7916B98F8D99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{185E7927-55DF-B544-BA77-C3C9E03ED088}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{185E7927-55DF-B544-BA77-C3C9E03ED088}"/>
   </bookViews>
   <sheets>
     <sheet name="Weekly Period Plan" sheetId="4" r:id="rId1"/>
@@ -435,7 +435,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -495,6 +495,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1476,55 +1479,55 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="1:13" s="22" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="22">
         <f>SUM(B3:B17)</f>
         <v>42</v>
       </c>
-      <c r="C18">
+      <c r="C18" s="22">
         <f t="shared" ref="C18:M18" si="0">SUM(C3:C17)</f>
         <v>42</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="E18">
+      <c r="E18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="G18">
+      <c r="G18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="H18">
+      <c r="H18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="I18">
+      <c r="I18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="J18">
+      <c r="J18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="L18">
+      <c r="L18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>
-      <c r="M18">
+      <c r="M18" s="22">
         <f t="shared" si="0"/>
         <v>42</v>
       </c>

</xml_diff>